<commit_message>
Busca no navegador, CEP, clima, postos, WhatsApp/QR, nova roteirizacao
</commit_message>
<xml_diff>
--- a/app/static/modelo_pontos.xlsx
+++ b/app/static/modelo_pontos.xlsx
@@ -492,9 +492,6 @@
           <t>sim</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -510,9 +507,6 @@
       <c r="C3" t="n">
         <v>100</v>
       </c>
-      <c r="D3" t="inlineStr"/>
-      <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr"/>
       <c r="G3" t="n">
         <v>5</v>
       </c>
@@ -531,9 +525,6 @@
       <c r="C4" t="n">
         <v>80</v>
       </c>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr"/>
       <c r="G4" t="n">
         <v>5</v>
       </c>
@@ -552,9 +543,6 @@
       <c r="C5" t="n">
         <v>70</v>
       </c>
-      <c r="D5" t="inlineStr"/>
-      <c r="E5" t="inlineStr"/>
-      <c r="F5" t="inlineStr"/>
       <c r="G5" t="n">
         <v>5</v>
       </c>
@@ -573,9 +561,6 @@
       <c r="C6" t="n">
         <v>80</v>
       </c>
-      <c r="D6" t="inlineStr"/>
-      <c r="E6" t="inlineStr"/>
-      <c r="F6" t="inlineStr"/>
       <c r="G6" t="n">
         <v>5</v>
       </c>
@@ -594,9 +579,6 @@
       <c r="C7" t="n">
         <v>100</v>
       </c>
-      <c r="D7" t="inlineStr"/>
-      <c r="E7" t="inlineStr"/>
-      <c r="F7" t="inlineStr"/>
       <c r="G7" t="n">
         <v>5</v>
       </c>
@@ -615,9 +597,6 @@
       <c r="C8" t="n">
         <v>50</v>
       </c>
-      <c r="D8" t="inlineStr"/>
-      <c r="E8" t="inlineStr"/>
-      <c r="F8" t="inlineStr"/>
       <c r="G8" t="n">
         <v>5</v>
       </c>
@@ -636,9 +615,6 @@
       <c r="C9" t="n">
         <v>60</v>
       </c>
-      <c r="D9" t="inlineStr"/>
-      <c r="E9" t="inlineStr"/>
-      <c r="F9" t="inlineStr"/>
       <c r="G9" t="n">
         <v>5</v>
       </c>
@@ -654,7 +630,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A7"/>
+  <dimension ref="A1:A8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -709,6 +685,13 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Opcional: em vez do endereço, informe as colunas cep e numero (o endereço é preenchido pelo ViaCEP).</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>